<commit_message>
docs: Lab 6 drafts the Pareto-chart skill in Microsoft 365 Copilot web
Lab 6 now sends learners to https://copilot.cloud.microsoft/ (the same
link Lab 8 uses) to draft the pareto-chart SKILL.md, and labels its web
prompts "Microsoft 365 Copilot web". Deck, Learner Guide, Lesson Plan,
labs and prompts page rebuilt; .gitignore now excludes *.zip and
**/reference/.

Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/labs/lab-06-custom-skills-pareto-chart/data/BrightPath_Job_Postings.xlsx
+++ b/labs/lab-06-custom-skills-pareto-chart/data/BrightPath_Job_Postings.xlsx
@@ -17287,7 +17287,7 @@
       </c>
       <c r="B2" s="5" t="inlineStr">
         <is>
-          <t>Microsoft Copilot web</t>
+          <t>Microsoft 365 Copilot web</t>
         </is>
       </c>
       <c r="C2" s="5" t="inlineStr">
@@ -17386,7 +17386,7 @@
       </c>
       <c r="B7" s="5" t="inlineStr">
         <is>
-          <t>Microsoft Copilot web</t>
+          <t>Microsoft 365 Copilot web</t>
         </is>
       </c>
       <c r="C7" s="5" t="inlineStr">
@@ -17443,7 +17443,7 @@
       </c>
       <c r="C10" s="5" t="inlineStr">
         <is>
-          <t>In the web chat at https://copilot.microsoft.com, use the complete Step 2 prompt below to draft pareto-chart. It describes the table, columns and chart because the web chat cannot see your workbook.</t>
+          <t>In the web chat at https://copilot.cloud.microsoft/, use the complete Step 2 prompt below to draft pareto-chart. It describes the table, columns and chart because the web chat cannot see your workbook.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Release C34 v3.2 with consistent Pareto skill rerun instructions
</commit_message>
<xml_diff>
--- a/labs/lab-06-custom-skills-pareto-chart/data/BrightPath_Job_Postings.xlsx
+++ b/labs/lab-06-custom-skills-pareto-chart/data/BrightPath_Job_Postings.xlsx
@@ -17298,8 +17298,9 @@
 Description: Use when I ask for a Pareto chart, an 80/20 analysis or the vital few categories in a table column.
 When the skill runs in Excel I will name a table and a category column, for example tblJobs and Job_Category. If I do not, it must ask me.
 Steps:
-1) Never change the source table or any existing sheet.
-2) Create a new sheet named Pareto_&lt;column name&gt; with a summary table: Category, Count, Share %, Cumulative %, sorted by Count from highest to lowest. Use formulas that read the source table so it updates when rows are added, and add a Total row.
+1) Never change the source table or unrelated sheets. You may replace only the matching Pareto_&lt;column name&gt; output sheet when rerunning this skill.
+2) Create a sheet named Pareto_&lt;column name&gt;; if it already exists, replace only its contents.
+Build a summary table: Category, Count, Share %, Cumulative %, sorted by Count from highest to lowest. Use formulas that read the source table so it updates when rows are added, and add a Total row.
 3) Create one combo chart from the summary: Count as columns and Cumulative % as a line with markers on a secondary axis from 0% to 100%.
 4) Give every column a different colour. Never use one colour for all the columns. Make the line dark grey.
 5) Format the chart cleanly: white background, no border or effects, data labels on the columns, axis titles, no legend, and a title that states the finding, for example "6 of 16 categories make up 83% of the total".

</xml_diff>